<commit_message>
fix: la dedicatoria dejó de personalizarse al renombrar el marcador
El texto pasó a "Hemos reservado N lugares en tu honor" y con él el atributo
data-invitado="pases" se renombró a "lugares". El JavaScript buscaba "pases",
así que no encontraba el hueco: todos los invitados habrían visto el número
escrito a mano en vez del suyo.

Ahora entiende las dos palabras, cada una con su singular: "1 pase"/"N pases"
y "1 lugar"/"N lugares".

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S7SFSJd7oRhveKMHswiAoK
</commit_message>
<xml_diff>
--- a/invitados y pases.xlsx
+++ b/invitados y pases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josep\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\~JORDANRM\Pictures\Proyectos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D4A2693-5216-4103-A68E-FB4846D3C2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E000014C-CC63-4440-A02A-1101F27FE360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{EBEC648F-ED95-4BC3-A7C0-5F1E1F8A6A67}"/>
+    <workbookView xWindow="2928" yWindow="2928" windowWidth="17280" windowHeight="8880" xr2:uid="{EBEC648F-ED95-4BC3-A7C0-5F1E1F8A6A67}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,17 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -33,9 +44,6 @@
     <t>pases</t>
   </si>
   <si>
-    <t>Sr. José Pedro Román Paladines y Esposa</t>
-  </si>
-  <si>
     <t>Sra. Sofia Encarnación</t>
   </si>
   <si>
@@ -54,9 +62,6 @@
     <t xml:space="preserve">Sr. Carlos Román </t>
   </si>
   <si>
-    <t>Sr. Jordan Román</t>
-  </si>
-  <si>
     <t>Sr. Franco Román y Esposa</t>
   </si>
   <si>
@@ -112,14 +117,28 @@
   </si>
   <si>
     <t>Sr. Ramiro Córdova y Esposa</t>
+  </si>
+  <si>
+    <t>Sr. José Pedro Román y Esposa</t>
+  </si>
+  <si>
+    <t>Lic. Jordan Román</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -147,8 +166,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -167,9 +187,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -207,7 +227,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -313,7 +333,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -455,7 +475,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -463,13 +483,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCA626D4-2ED9-4EBF-A2A2-552787A59FAF}">
-  <dimension ref="A1:B28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.42578125" customWidth="1"/>
+    <col min="1" max="1" width="39.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -477,221 +497,224 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="B2">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>3</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
       </c>
       <c r="B4">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
       <c r="B10">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>11</v>
       </c>
-      <c r="B12">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="B14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>12</v>
       </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="B15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>14</v>
       </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>26</v>
-      </c>
-      <c r="B16">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="B19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>18</v>
-      </c>
-      <c r="B18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>17</v>
-      </c>
-      <c r="B20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>20</v>
       </c>
       <c r="B22">
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>21</v>
       </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="B25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>22</v>
       </c>
-      <c r="B24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="B26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>23</v>
       </c>
-      <c r="B25">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>24</v>
-      </c>
-      <c r="B26">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>25</v>
-      </c>
       <c r="B27">
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B28">
         <v>2</v>
       </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B29" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>